<commit_message>
ace fix and brazil europe
</commit_message>
<xml_diff>
--- a/content/economics/ACE_landing_page_data.xlsx
+++ b/content/economics/ACE_landing_page_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\oaolive\repos\aiu-portal\content\economics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8254106-DBCF-432D-BC27-E34568B91154}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB72482F-7259-4004-80A1-6DBD357F8BD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="18240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ACE_landing_page_data" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
   <si>
     <t>year_data</t>
   </si>
@@ -195,10 +195,7 @@
     <t>HASP</t>
   </si>
   <si>
-    <t>UkSATSE</t>
-  </si>
-  <si>
-    <t>AirNav Ireland</t>
+    <t>Airnav Ireland</t>
   </si>
 </sst>
 </file>
@@ -1144,46 +1141,46 @@
         <v>2024</v>
       </c>
       <c r="B2">
-        <v>469.4605934329557</v>
+        <v>469.39225682651136</v>
       </c>
       <c r="C2">
-        <v>10467653125.780624</v>
+        <v>10466091408.836081</v>
       </c>
       <c r="D2">
-        <v>22297192.293042853</v>
+        <v>22297111.331992798</v>
       </c>
       <c r="E2">
-        <v>0.98081881913019253</v>
+        <v>0.98079204699871292</v>
       </c>
       <c r="F2">
-        <v>152.18400188546104</v>
+        <v>152.82398138891722</v>
       </c>
       <c r="G2">
-        <v>314.30043651384142</v>
+        <v>313.57535164608248</v>
       </c>
       <c r="H2">
-        <v>-1.3990770346900772E-2</v>
+        <v>-1.4071130843755331E-2</v>
       </c>
       <c r="I2">
-        <v>4.0218364367912596E-2</v>
+        <v>4.0148961400319205E-2</v>
       </c>
       <c r="J2">
-        <v>5.4978323817399977E-2</v>
+        <v>5.4993918872135117E-2</v>
       </c>
       <c r="K2">
-        <v>4.7861539125722885E-2</v>
+        <v>4.7132165954537175E-2</v>
       </c>
       <c r="L2">
-        <v>3.8514105249225938E-2</v>
+        <v>3.813057254531671E-2</v>
       </c>
       <c r="M2">
-        <v>-1.6474730305083396E-2</v>
+        <v>-1.6769109182996123E-2</v>
       </c>
       <c r="N2">
-        <v>100.98603190277626</v>
+        <v>100.97096533577317</v>
       </c>
       <c r="O2">
-        <v>102.09317864913423</v>
+        <v>102.09468528277846</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
@@ -1191,46 +1188,46 @@
         <v>2023</v>
       </c>
       <c r="B3">
-        <v>476.12190567234626</v>
+        <v>476.0914012267599</v>
       </c>
       <c r="C3">
-        <v>10062938210.229813</v>
+        <v>10062108214.52527</v>
       </c>
       <c r="D3">
-        <v>21135213.671842363</v>
+        <v>21134824.507642683</v>
       </c>
       <c r="E3">
-        <v>0.93601948588411121</v>
+        <v>0.93664589713434077</v>
       </c>
       <c r="F3">
-        <v>146.54013952842695</v>
+        <v>147.21075116227357</v>
       </c>
       <c r="G3">
-        <v>319.56518678095119</v>
+        <v>318.92341318275794</v>
       </c>
       <c r="H3">
-        <v>-7.2964061904103206E-2</v>
+        <v>-7.3039848706425992E-2</v>
       </c>
       <c r="I3">
-        <v>2.9726379638513656E-2</v>
+        <v>2.9641447340004179E-2</v>
       </c>
       <c r="J3">
-        <v>0.11077288088047554</v>
+        <v>0.11077207138099543</v>
       </c>
       <c r="K3">
-        <v>8.8513539388441087E-2</v>
+        <v>8.9261266896878411E-2</v>
       </c>
       <c r="L3">
-        <v>2.1614143908957439E-2</v>
+        <v>2.3706116256983378E-2</v>
       </c>
       <c r="M3">
-        <v>-7.8497934256253843E-2</v>
+        <v>-7.9247219516262568E-2</v>
       </c>
       <c r="N3">
-        <v>97.081569949152268</v>
+        <v>97.073562617261274</v>
       </c>
       <c r="O3">
-        <v>96.772773756823597</v>
+        <v>96.772771346326863</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
@@ -1238,46 +1235,46 @@
         <v>2022</v>
       </c>
       <c r="B4">
-        <v>513.59595254773615</v>
+        <v>513.60503529992502</v>
       </c>
       <c r="C4">
         <v>9772438979.1416397</v>
       </c>
       <c r="D4">
-        <v>19027484.408053901</v>
+        <v>19027147.920064535</v>
       </c>
       <c r="E4">
-        <v>0.85990614908657403</v>
+        <v>0.85989094223710616</v>
       </c>
       <c r="F4">
-        <v>143.43981081519371</v>
+        <v>143.80176969199519</v>
       </c>
       <c r="G4">
-        <v>346.78727119621755</v>
+        <v>346.37246820498831</v>
       </c>
       <c r="H4">
-        <v>-0.34491825017192079</v>
+        <v>-0.3449185827401875</v>
       </c>
       <c r="I4">
-        <v>3.6839780409229528E-2</v>
+        <v>3.6839780409229306E-2</v>
       </c>
       <c r="J4">
-        <v>0.58276395378338597</v>
+        <v>0.58276475731261246</v>
       </c>
       <c r="K4">
-        <v>0.42197440293200161</v>
+        <v>0.4262610245536711</v>
       </c>
       <c r="L4">
-        <v>-3.3503681179227307E-2</v>
+        <v>-3.1369659813227702E-2</v>
       </c>
       <c r="M4">
-        <v>-0.35612961410659494</v>
+        <v>-0.35593426581459786</v>
       </c>
       <c r="N4">
-        <v>94.278996701272078</v>
+        <v>94.278996701272092</v>
       </c>
       <c r="O4">
-        <v>87.122016951039342</v>
+        <v>87.122078273008498</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
@@ -1285,46 +1282,46 @@
         <v>2021</v>
       </c>
       <c r="B5">
-        <v>784.01810565250082</v>
+        <v>784.03236875245329</v>
       </c>
       <c r="C5">
-        <v>9425216088.144846</v>
+        <v>9425216088.1448479</v>
       </c>
       <c r="D5">
-        <v>12021681.668053685</v>
+        <v>12021462.96987991</v>
       </c>
       <c r="E5">
-        <v>0.6047268834892624</v>
+        <v>0.60289871729909839</v>
       </c>
       <c r="F5">
-        <v>148.41216466318815</v>
+        <v>148.45887406775549</v>
       </c>
       <c r="G5">
-        <v>538.59795200090059</v>
+        <v>537.79055431829693</v>
       </c>
       <c r="H5">
-        <v>-0.25272924176920852</v>
+        <v>-0.25272955306053124</v>
       </c>
       <c r="I5">
-        <v>-4.9774400373029382E-2</v>
+        <v>-4.977440037302916E-2</v>
       </c>
       <c r="J5">
-        <v>0.27159478563925998</v>
+        <v>0.27159531534898518</v>
       </c>
       <c r="K5">
-        <v>0.25213414892893815</v>
+        <v>0.25003589688951244</v>
       </c>
       <c r="L5">
-        <v>-8.2604403998122189E-2</v>
+        <v>-8.0912879580180341E-2</v>
       </c>
       <c r="M5">
-        <v>-0.24587929212811932</v>
+        <v>-0.2470928166228904</v>
       </c>
       <c r="N5">
-        <v>90.929185475562264</v>
+        <v>90.929185475562292</v>
       </c>
       <c r="O5">
-        <v>55.044226110144713</v>
+        <v>55.044236909175105</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
@@ -1332,46 +1329,46 @@
         <v>2020</v>
       </c>
       <c r="B6">
-        <v>1049.1754120135931</v>
+        <v>1049.1949360014801</v>
       </c>
       <c r="C6">
         <v>9918924613.1075573</v>
       </c>
       <c r="D6">
-        <v>9454019.3179622926</v>
+        <v>9453843.3924480602</v>
       </c>
       <c r="E6">
-        <v>0.48295694515363163</v>
+        <v>0.48230512323630259</v>
       </c>
       <c r="F6">
-        <v>161.77553643159669</v>
+        <v>161.52861983306065</v>
       </c>
       <c r="G6">
-        <v>714.20655390940976</v>
+        <v>714.28532784888182</v>
       </c>
       <c r="H6">
-        <v>1.210617188802134</v>
+        <v>1.2106176759843055</v>
       </c>
       <c r="I6">
-        <v>-4.3077922640073374E-2</v>
+        <v>-4.3077922640073263E-2</v>
       </c>
       <c r="J6">
-        <v>-0.56712447446477454</v>
+        <v>-0.56712456986310622</v>
       </c>
       <c r="K6">
-        <v>-0.50708837746858282</v>
+        <v>-0.50626881861211737</v>
       </c>
       <c r="L6">
-        <v>8.3696161698424421E-2</v>
+        <v>8.5286049846981182E-2</v>
       </c>
       <c r="M6">
-        <v>1.2163174140894872</v>
+        <v>1.2165211059548868</v>
       </c>
       <c r="N6">
         <v>95.692207735992667</v>
       </c>
       <c r="O6">
-        <v>43.287552553522552</v>
+        <v>43.287543013689387</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
@@ -1379,40 +1376,40 @@
         <v>2019</v>
       </c>
       <c r="B7">
-        <v>474.60746135883858</v>
+        <v>474.61618867871977</v>
       </c>
       <c r="C7">
-        <v>10365446516.265041</v>
+        <v>10365446516.265039</v>
       </c>
       <c r="D7">
-        <v>21840041.213401809</v>
+        <v>21839639.615162145</v>
       </c>
       <c r="E7">
-        <v>0.97980433626891994</v>
+        <v>0.97685773436577106</v>
       </c>
       <c r="F7">
-        <v>149.2812673416262</v>
+        <v>148.83506505573826</v>
       </c>
       <c r="G7">
-        <v>322.2492181711354</v>
+        <v>322.25514385127616</v>
       </c>
       <c r="H7">
-        <v>-2.3237134232800827E-3</v>
+        <v>-2.324023302582634E-3</v>
       </c>
       <c r="I7">
         <v>1.4159414678369009E-2</v>
       </c>
       <c r="J7">
-        <v>1.6521519378000837E-2</v>
+        <v>1.6521835110750338E-2</v>
       </c>
       <c r="K7">
-        <v>1.0339197903164399E-2</v>
+        <v>7.3196030045683536E-3</v>
       </c>
       <c r="L7">
-        <v>5.633255473421972E-3</v>
+        <v>2.6274137804365161E-3</v>
       </c>
       <c r="M7">
-        <v>-1.2163576101731355E-3</v>
+        <v>-1.2166678334214476E-3</v>
       </c>
       <c r="N7">
         <v>100</v>
@@ -1428,7 +1425,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:A40"/>
+  <dimension ref="A1:A39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="19.140625" bestFit="1" customWidth="1"/>
@@ -1441,7 +1438,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
@@ -1620,18 +1617,13 @@
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A38" s="3" t="s">
+      <c r="A38" s="4" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A39" s="4" t="s">
+      <c r="A39" s="5" t="s">
         <v>50</v>
-      </c>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A40" s="5" t="s">
-        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>